<commit_message>
Fix matching: align R-ID file dates with collection log + fix button truncation
[매칭 수정]
- R-ID 파일 방문일을 수집일지 최신 접수일자와 일치하도록 전면 수정
  → 매칭 성공 8건, 미매칭 1건(정자차 성별 오기입 데모용)
- 정자차 개인번호 M01.09 → F01.09 (오기입 시뮬레이션)
  → feature 4(수집관리시스템 보정)에서 남으로 보정 후 매칭 복구

[수집관리시스템 샘플 수정]
- 10005(정자차): 남으로 보정 (기존 유지)
- 10008(윤거너) → 10014(나도현): 더 명확한 보정 케이스로 교체

[UI 수정]
- 발송 대상 선택 다이얼로그 260→360px, 버튼 width 10→14 (한글 잘림 수정)
- 미매칭 시트 없을 때 구체적 안내 메시지 추가

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sample_data/rid_파일_샘플.xlsx
+++ b/sample_data/rid_파일_샘플.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="43">
   <si>
     <t>환자ID</t>
   </si>
@@ -49,22 +49,40 @@
     <t>RID-2024-006</t>
   </si>
   <si>
+    <t>RID-2024-007</t>
+  </si>
+  <si>
+    <t>RID-2024-008</t>
+  </si>
+  <si>
+    <t>RID-2024-009</t>
+  </si>
+  <si>
     <t>김가나</t>
   </si>
   <si>
     <t>이다라</t>
   </si>
   <si>
+    <t>최사아</t>
+  </si>
+  <si>
+    <t>강카타</t>
+  </si>
+  <si>
+    <t>조파하</t>
+  </si>
+  <si>
+    <t>한서연</t>
+  </si>
+  <si>
+    <t>임도영</t>
+  </si>
+  <si>
     <t>박마바</t>
   </si>
   <si>
-    <t>최사아</t>
-  </si>
-  <si>
-    <t>강카타</t>
-  </si>
-  <si>
-    <t>조파하</t>
+    <t>정자차</t>
   </si>
   <si>
     <t>남</t>
@@ -79,25 +97,52 @@
     <t>1975-11</t>
   </si>
   <si>
+    <t>1990-04</t>
+  </si>
+  <si>
+    <t>1955-12</t>
+  </si>
+  <si>
+    <t>1979-06</t>
+  </si>
+  <si>
+    <t>1988-08</t>
+  </si>
+  <si>
+    <t>1971-03</t>
+  </si>
+  <si>
     <t>1982-07</t>
   </si>
   <si>
-    <t>1990-04</t>
-  </si>
-  <si>
-    <t>1955-12</t>
-  </si>
-  <si>
-    <t>1979-06</t>
-  </si>
-  <si>
-    <t>2024-03-15</t>
-  </si>
-  <si>
-    <t>2024-03-16</t>
-  </si>
-  <si>
-    <t>2024-03-17</t>
+    <t>2001-09</t>
+  </si>
+  <si>
+    <t>2024-06-10</t>
+  </si>
+  <si>
+    <t>2024-06-15</t>
+  </si>
+  <si>
+    <t>2024-06-20</t>
+  </si>
+  <si>
+    <t>2024-07-08</t>
+  </si>
+  <si>
+    <t>2024-07-15</t>
+  </si>
+  <si>
+    <t>2024-04-18</t>
+  </si>
+  <si>
+    <t>2024-07-05</t>
+  </si>
+  <si>
+    <t>2024-07-10</t>
+  </si>
+  <si>
+    <t>2024-07-01</t>
   </si>
 </sst>
 </file>
@@ -429,7 +474,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -454,16 +499,16 @@
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C2" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="D2" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="E2" t="s">
-        <v>25</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -471,16 +516,16 @@
         <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="C3" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="D3" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="E3" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -488,16 +533,16 @@
         <v>7</v>
       </c>
       <c r="B4" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="C4" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="D4" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="E4" t="s">
-        <v>25</v>
+        <v>36</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -505,16 +550,16 @@
         <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C5" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="D5" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="E5" t="s">
-        <v>26</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -522,16 +567,16 @@
         <v>9</v>
       </c>
       <c r="B6" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C6" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="D6" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="E6" t="s">
-        <v>27</v>
+        <v>38</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -539,16 +584,67 @@
         <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C7" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="D7" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="E7" t="s">
-        <v>27</v>
+        <v>39</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8" t="s">
+        <v>23</v>
+      </c>
+      <c r="D8" t="s">
+        <v>31</v>
+      </c>
+      <c r="E8" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" t="s">
+        <v>21</v>
+      </c>
+      <c r="C9" t="s">
+        <v>23</v>
+      </c>
+      <c r="D9" t="s">
+        <v>32</v>
+      </c>
+      <c r="E9" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10" t="s">
+        <v>22</v>
+      </c>
+      <c r="C10" t="s">
+        <v>23</v>
+      </c>
+      <c r="D10" t="s">
+        <v>33</v>
+      </c>
+      <c r="E10" t="s">
+        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>